<commit_message>
feat: change in handling outlier IQR
</commit_message>
<xml_diff>
--- a/losers.xlsx
+++ b/losers.xlsx
@@ -413,428 +413,204 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>24h Change</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>24h Change</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t>Volume(24h)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>siren84SIREN</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>siren81SIREN</t>
+          <t>$0.7112</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>$0.7006</t>
+          <t>65.83%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>65.66%</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>$177,523,169</t>
+          <t>$166,076,225</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Worldcoin61WLD</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Worldcoin62WLD</t>
+          <t>$0.2872</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>$0.2816</t>
+          <t>9.87%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11.39%</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>$305,768,614</t>
+          <t>$308,351,768</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Algorand57ALGO</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Algorand57ALGO</t>
+          <t>$0.1116</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>$0.1107</t>
+          <t>2.60%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.39%</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>$53,919,285</t>
+          <t>$53,182,799</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Toncoin30TON</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Toncoin30TON</t>
+          <t>$1.40</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>$1.40</t>
+          <t>2.58%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.03%</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>$156,133,045</t>
+          <t>$151,353,430</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PancakeSwap83CAKE</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PancakeSwap83CAKE</t>
+          <t>$1.59</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>$1.58</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.57%</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>$61,843,569</t>
+          <t>$61,753,770</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>UNUS SED LEO11LEO</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OFFICIAL TRUMP70TRUMP</t>
+          <t>$10.14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$2.99</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.44%</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>$183,383,858</t>
+          <t>$524,198</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Canton20CC</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Artificial Superintelligence Alliance82FET</t>
+          <t>$0.1486</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>$0.2292</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.01%</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>$199,544,463</t>
+          <t>$12,642,674</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NEAR Protocol42NEAR</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Stacks91STX</t>
+          <t>$1.42</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>$0.2381</t>
+          <t>0.02%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.00%</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>$20,341,360</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>LayerZero76ZRO</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>$1.94</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>0.70%</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>$42,483,384</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>XDC Network74XDC</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>$0.03109</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>0.67%</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>$26,255,450</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>VeChain73VET</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>$0.007236</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0.52%</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>$24,382,797</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>NEAR Protocol42NEAR</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>$1.40</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>0.52%</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>$272,745,339</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>World Liberty Financial34WLFI</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>$0.08064</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>0.45%</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>$103,939,325</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Venice Token95VVV</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>$8.93</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>0.34%</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>$22,407,761</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Render59RENDER</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>$1.86</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>0.18%</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>$106,598,424</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Filecoin68FIL</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>$0.9781</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>0.02%</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>$158,332,611</t>
+          <t>$272,469,032</t>
         </is>
       </c>
     </row>

</xml_diff>